<commit_message>
added UI todolist app to my git repo
</commit_message>
<xml_diff>
--- a/MyToDoList.xlsx
+++ b/MyToDoList.xlsx
@@ -10,7 +10,7 @@
     <sheet name="TaskSubTask" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todo List'!$A$1:$J$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todo List'!$A$1:$J$48</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1301,674 +1301,730 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>b201e0936e8f4aa99e975174b420f4b9</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Pune List</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Bills</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Airtel postpaid mobile bill</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>2026-08-20 11:44:48</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:25</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>35def8a789dc4f26ab97505ce874f168</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Pune List</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Bills</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>RD E2107 Ebill</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>2026-08-20 11:44:48</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:25</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>1e17d7a989e847d58777c2e73b75ee2b</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Gaya List</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Bills</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Gaya Papa Ebills</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>2026-08-20 11:44:48</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>4373b66ab906478792d19704e0f6c8a7</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Gaya List</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Bills</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Gaya Renters Ebills</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>2026-08-20 11:44:48</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>3547cb63adf7447c9461e76efa67fd08</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Pune List</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Creditcard bills</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Amazonpay ICICI</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>2026-08-20 11:44:54</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>0d9f1ffdd02349c4bdf92ff722eae70f</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Pune List</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Creditcard bills</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Tata Neu HDFC</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>2026-08-20 11:44:54</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>8d291a1265234345b4b3b6a05fb0f8b0</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Pune List</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Creditcard bills</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Swiggy HDFC</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>2026-08-20 11:44:54</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>f0926ca829dc45d7b72491bf42ce39e2</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Pune List</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Creditcard bills</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Rupay UPI CC HDFC</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>2026-08-20 11:44:54</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>be8b06355bf74ea08802ea512fc829b7</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Pune List</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Creditcard bills</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Regalia Gold HDFC</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>2026-08-20 11:44:54</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>7c7c5248236144c4ae2dd2eee19fb283</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Pune List</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Creditcard bills</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Airtel AXIS</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>2026-08-20 11:44:54</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>e01767a73a8e4d1bafeb4be3c89b81f5</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Pune List</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Creditcard bills</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>KIWI YesBank</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>2026-08-20 11:44:54</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>db3bc4013cce41ba84ba1c86de3250c1</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Pune List</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>EMIs</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>Home Loan EMI</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>2026-08-20 11:45:01</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:36</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>a27dfa595de04355999d58741f44cc39</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Pune List</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>EMIs</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>Car Loan EMI</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>2026-08-20 11:45:01</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:36</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>0ff8ac886b94410eb04f1b04ba3d0c26</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Pune List</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Fees</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>Aarya School Fee</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>Quarterly</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>OCT</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>2026-10</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>2026-08-20 11:45:05</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>2026-AUG-20</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2020,10 +2076,838 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>70bb96a162a94f0c8295c683e02ccae1</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Airtel postpaid mobile bill</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:25</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>2026-AUG-20</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>3e447e81bbfe4b1980f6456624c33710</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>RD E2107 Ebill</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:25</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>6fa01b168c4a4616b9d1632472168655</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Gaya List</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Gaya Papa Ebills</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>900bacce9a7841d1994433ac2adbbc3b</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Gaya List</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Gaya Renters Ebills</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>2026-AUG-20</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>7d731e9b708d4b7a9cb1a2d48e99b874</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Creditcard bills</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Amazonpay ICICI</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>9fa67d5c276149fd91afa1cb018f0614</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Creditcard bills</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Tata Neu HDFC</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>69102eb9dd1f436ea511f0797b2340ed</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Creditcard bills</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Swiggy HDFC</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>17a5960e0c904c3b80a3b8c2a4f03e52</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Creditcard bills</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Rupay UPI CC HDFC</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2857f61a984a4e6bbe28b654ec04424f</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Creditcard bills</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Regalia Gold HDFC</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>46b26cb529974fceb8c4479384c1f4c2</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Creditcard bills</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Airtel AXIS</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>3efb743ef1e849efbd789651e979d30d</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Creditcard bills</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>KIWI YesBank</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:28</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>5ebf570c13ae4d8db7737765a1d3d62f</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>EMIs</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Home Loan EMI</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:36</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>b973cdf545724b04937b50363d01d691</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>EMIs</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Car Loan EMI</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2026-08-20 12:58:36</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ca50f636b92548bab6ee0a2f565c25fe</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Fees</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Aarya School Fee</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>JAN</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2026-08-20 13:55:27</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>b10e3caf10e54fc7b7a7c1ec6daa633e</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Airtel postpaid mobile bill</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>OCT</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20 13:55:53</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>2026-AUG-20</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>4e365162d46b4d818a3d2ec1731fa333</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Gaya List</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Gaya Renters Ebills</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>OCT</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-08-20 14:01:21</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>13208cb0d5624926aaf205cdb7f4a882</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Pune List</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Airtel postpaid mobile bill</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>NOV</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>2026-08-20 14:05:43</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J31"/>
+  <autoFilter ref="A1:J48"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="J2:J48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pending,Done"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>